<commit_message>
Sync Adult notebook metrics into the dashboard.
Extract latest Adult SDV fidelity/privacy tables from the notebook, update MasterData and docs/data JSON, harden HTML table parsing and MetricValue export, and speed up Gower with an 800-row subsample.
</commit_message>
<xml_diff>
--- a/paper results/3. Adult/TRTR_TSTR_results_adult.xlsx
+++ b/paper results/3. Adult/TRTR_TSTR_results_adult.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="TRTR_Results" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="All_Comparisons" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="CTGAN" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="CopulaGAN" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TVAE" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="GaussianCopula" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="WGAN_GP" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="CTABGAN" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="TabDDPM" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="ForestDiffusion" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRTR_Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All_Comparisons" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CTGAN" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CopulaGAN" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TVAE" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GaussianCopula" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WGAN_GP" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CTABGAN" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TabDDPM" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ForestDiffusion" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,13 +27,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -44,7 +47,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -52,12 +55,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,87 +439,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>F1 Std</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Precision Std</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Recall Std</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)</t>
         </is>
@@ -1238,192 +1250,192 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Accuracy_Drop</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>F1_Drop</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Precision_Drop</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Recall_Drop</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -2964,192 +2976,192 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Accuracy_Drop</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>F1_Drop</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Precision_Drop</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Recall_Drop</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -4690,192 +4702,192 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Accuracy_Drop</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>F1_Drop</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Precision_Drop</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Recall_Drop</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -17056,27 +17068,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Accuracy_Drop</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>F1_Drop</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Precision_Drop</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Recall_Drop</t>
         </is>
@@ -17249,192 +17261,192 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Accuracy_Drop</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>F1_Drop</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Precision_Drop</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Recall_Drop</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -18975,192 +18987,192 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Accuracy_Drop</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>F1_Drop</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Precision_Drop</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Recall_Drop</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -20701,192 +20713,192 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Accuracy_Drop</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>F1_Drop</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Precision_Drop</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Recall_Drop</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -22427,192 +22439,192 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Accuracy_Drop</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>F1_Drop</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Precision_Drop</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Recall_Drop</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -24153,192 +24165,192 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Accuracy_Drop</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>F1_Drop</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Precision_Drop</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Recall_Drop</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>
@@ -25879,192 +25891,192 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TRTR</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TRTR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TRTR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TRTR</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TRTR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TRTR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TRTR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TRTR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TRTR</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TRTR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TRTR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TRTR</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TRTR</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Mean_TSTR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Accuracy Std_TSTR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>F1 Mean_TSTR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>F1 Std_TSTR</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Precision Mean_TSTR</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Precision Std_TSTR</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Recall Mean_TSTR</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Recall Std_TSTR</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Accuracy ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>F1 ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Precision ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Recall ± SD_TSTR</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Accuracy (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>F1 (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Precision (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Recall (Mean±Std)_TSTR</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Accuracy_Drop</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>F1_Drop</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Precision_Drop</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Recall_Drop</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Synthetic_Model</t>
         </is>

</xml_diff>